<commit_message>
simplify calendar match labels
</commit_message>
<xml_diff>
--- a/outputs/wc2026_calendar/calendar_chm_2026_msk.xlsx
+++ b/outputs/wc2026_calendar/calendar_chm_2026_msk.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Календарь" sheetId="1" r:id="Rb6ed1ac9aa254fec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Список МСК" sheetId="2" r:id="R05feb48d79d84710"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мой выбор" sheetId="3" r:id="R985726e7fe1d4ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все матчи" sheetId="4" r:id="R695f85dc68574f00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="5" r:id="R03d7c72f5c064b8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Стадионы" sheetId="6" r:id="R42afc6565b8f4bd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источник" sheetId="7" r:id="Rb0b84cba1b064adb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Календарь" sheetId="1" r:id="R4bc2d3d4ceea474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Список МСК" sheetId="2" r:id="Re78f1a6290cc47f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мой выбор" sheetId="3" r:id="Rb715d31fe4654bae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все матчи" sheetId="4" r:id="Rb627cbb6d9994c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Группы" sheetId="5" r:id="Rf526f65763e549e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Стадионы" sheetId="6" r:id="R32e9c0b542c04ca8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источник" sheetId="7" r:id="R4bb8117728fe4cc8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -644,7 +644,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb71b1ff9c05142a4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R33375b8907064e46"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1027,8 +1027,7 @@
       <x:c r="F8" s="77" t="str"/>
       <x:c r="G8" s="78" t="str"/>
       <x:c r="H8" s="79" t="str">
-        <x:v>Brazil - Morocco
-Группа C · #6</x:v>
+        <x:v>Бразилия - Марокко</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="43.5" customHeight="1">
@@ -1041,12 +1040,10 @@
       <x:c r="E9" s="77" t="str"/>
       <x:c r="F9" s="77" t="str"/>
       <x:c r="G9" s="79" t="str">
-        <x:v>USA - Paraguay
-Группа D · #4</x:v>
+        <x:v>США - Парагвай</x:v>
       </x:c>
       <x:c r="H9" s="79" t="str">
-        <x:v>Haiti - Scotland
-Группа C · #7</x:v>
+        <x:v>Гаити - Шотландия</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43.5" customHeight="1">
@@ -1058,8 +1055,7 @@
       <x:c r="D10" s="77" t="str"/>
       <x:c r="E10" s="77" t="str"/>
       <x:c r="F10" s="79" t="str">
-        <x:v>South Korea - Czechia
-Группа A · #2</x:v>
+        <x:v>Южная Корея - Чехия</x:v>
       </x:c>
       <x:c r="G10" s="78" t="str"/>
       <x:c r="H10" s="78" t="str"/>
@@ -1075,8 +1071,7 @@
       <x:c r="F11" s="77" t="str"/>
       <x:c r="G11" s="78" t="str"/>
       <x:c r="H11" s="79" t="str">
-        <x:v>Australia - Türkiye
-Группа D · #8</x:v>
+        <x:v>Австралия - Турция</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="43.5" customHeight="1">
@@ -1090,8 +1085,7 @@
       <x:c r="F12" s="77" t="str"/>
       <x:c r="G12" s="78" t="str"/>
       <x:c r="H12" s="79" t="str">
-        <x:v>Germany - Curaçao
-Группа E · #9</x:v>
+        <x:v>Германия - Кюрасао</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="43.5" customHeight="1">
@@ -1102,16 +1096,13 @@
       <x:c r="C13" s="77" t="str"/>
       <x:c r="D13" s="77" t="str"/>
       <x:c r="E13" s="79" t="str">
-        <x:v>Mexico - South Africa
-Группа A · #1</x:v>
+        <x:v>Мексика - ЮАР</x:v>
       </x:c>
       <x:c r="F13" s="79" t="str">
-        <x:v>Canada - Bosnia &amp; Herzegovina
-Группа B · #3</x:v>
+        <x:v>Канада - Босния и Герцеговина</x:v>
       </x:c>
       <x:c r="G13" s="79" t="str">
-        <x:v>Qatar - Switzerland
-Группа B · #5</x:v>
+        <x:v>Катар - Швейцария</x:v>
       </x:c>
       <x:c r="H13" s="78" t="str"/>
     </x:row>
@@ -1126,8 +1117,7 @@
       <x:c r="F14" s="77" t="str"/>
       <x:c r="G14" s="78" t="str"/>
       <x:c r="H14" s="79" t="str">
-        <x:v>Netherlands - Japan
-Группа F · #10</x:v>
+        <x:v>Нидерланды - Япония</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1232,21 +1222,17 @@
       </x:c>
       <x:c r="B20" s="77" t="str"/>
       <x:c r="C20" s="79" t="str">
-        <x:v>Saudi Arabia - Uruguay
-Группа H · #15</x:v>
+        <x:v>Саудовская Аравия - Уругвай</x:v>
       </x:c>
       <x:c r="D20" s="79" t="str">
-        <x:v>Iraq - Norway
-Группа I · #18</x:v>
+        <x:v>Ирак - Норвегия</x:v>
       </x:c>
       <x:c r="E20" s="77" t="str"/>
       <x:c r="F20" s="79" t="str">
-        <x:v>Canada - Qatar
-Группа B · #27</x:v>
+        <x:v>Канада - Катар</x:v>
       </x:c>
       <x:c r="G20" s="79" t="str">
-        <x:v>Scotland - Morocco
-Группа C · #30</x:v>
+        <x:v>Шотландия - Марокко</x:v>
       </x:c>
       <x:c r="H20" s="78" t="str"/>
     </x:row>
@@ -1255,14 +1241,12 @@
         <x:v>02:00</x:v>
       </x:c>
       <x:c r="B21" s="79" t="str">
-        <x:v>Ivory Coast - Ecuador
-Группа E · #11</x:v>
+        <x:v>Кот-д’Ивуар - Эквадор</x:v>
       </x:c>
       <x:c r="C21" s="77" t="str"/>
       <x:c r="D21" s="77" t="str"/>
       <x:c r="E21" s="79" t="str">
-        <x:v>Ghana - Panama
-Группа L · #23</x:v>
+        <x:v>Гана - Панама</x:v>
       </x:c>
       <x:c r="F21" s="77" t="str"/>
       <x:c r="G21" s="78" t="str"/>
@@ -1279,8 +1263,7 @@
       <x:c r="F22" s="77" t="str"/>
       <x:c r="G22" s="78" t="str"/>
       <x:c r="H22" s="79" t="str">
-        <x:v>Ecuador - Curaçao
-Группа E · #35</x:v>
+        <x:v>Эквадор - Кюрасао</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="43.5" customHeight="1">
@@ -1293,8 +1276,7 @@
       <x:c r="E23" s="77" t="str"/>
       <x:c r="F23" s="77" t="str"/>
       <x:c r="G23" s="79" t="str">
-        <x:v>Brazil - Haiti
-Группа C · #31</x:v>
+        <x:v>Бразилия - Гаити</x:v>
       </x:c>
       <x:c r="H23" s="78" t="str"/>
     </x:row>
@@ -1304,17 +1286,14 @@
       </x:c>
       <x:c r="B24" s="77" t="str"/>
       <x:c r="C24" s="79" t="str">
-        <x:v>Iran - New Zealand
-Группа G · #16</x:v>
+        <x:v>Иран - Новая Зеландия</x:v>
       </x:c>
       <x:c r="D24" s="79" t="str">
-        <x:v>Argentina - Algeria
-Группа J · #19</x:v>
+        <x:v>Аргентина - Алжир</x:v>
       </x:c>
       <x:c r="E24" s="77" t="str"/>
       <x:c r="F24" s="79" t="str">
-        <x:v>Mexico - South Korea
-Группа A · #28</x:v>
+        <x:v>Мексика - Южная Корея</x:v>
       </x:c>
       <x:c r="G24" s="78" t="str"/>
       <x:c r="H24" s="78" t="str"/>
@@ -1324,14 +1303,12 @@
         <x:v>05:00</x:v>
       </x:c>
       <x:c r="B25" s="79" t="str">
-        <x:v>Sweden - Tunisia
-Группа F · #12</x:v>
+        <x:v>Швеция - Тунис</x:v>
       </x:c>
       <x:c r="C25" s="77" t="str"/>
       <x:c r="D25" s="77" t="str"/>
       <x:c r="E25" s="79" t="str">
-        <x:v>Uzbekistan - Colombia
-Группа K · #24</x:v>
+        <x:v>Узбекистан - Колумбия</x:v>
       </x:c>
       <x:c r="F25" s="77" t="str"/>
       <x:c r="G25" s="78" t="str"/>
@@ -1347,8 +1324,7 @@
       <x:c r="E26" s="77" t="str"/>
       <x:c r="F26" s="77" t="str"/>
       <x:c r="G26" s="79" t="str">
-        <x:v>Türkiye - Paraguay
-Группа D · #32</x:v>
+        <x:v>Турция - Парагвай</x:v>
       </x:c>
       <x:c r="H26" s="78" t="str"/>
     </x:row>
@@ -1359,15 +1335,13 @@
       <x:c r="B27" s="77" t="str"/>
       <x:c r="C27" s="77" t="str"/>
       <x:c r="D27" s="79" t="str">
-        <x:v>Austria - Jordan
-Группа J · #20</x:v>
+        <x:v>Австрия - Иордания</x:v>
       </x:c>
       <x:c r="E27" s="77" t="str"/>
       <x:c r="F27" s="77" t="str"/>
       <x:c r="G27" s="78" t="str"/>
       <x:c r="H27" s="79" t="str">
-        <x:v>Tunisia - Japan
-Группа F · #36</x:v>
+        <x:v>Тунис - Япония</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="43.5" customHeight="1">
@@ -1375,20 +1349,17 @@
         <x:v>19:00</x:v>
       </x:c>
       <x:c r="B28" s="79" t="str">
-        <x:v>Spain - Cape Verde
-Группа H · #13</x:v>
+        <x:v>Испания - Кабо-Верде</x:v>
       </x:c>
       <x:c r="C28" s="77" t="str"/>
       <x:c r="D28" s="77" t="str"/>
       <x:c r="E28" s="79" t="str">
-        <x:v>Czechia - South Africa
-Группа A · #25</x:v>
+        <x:v>Чехия - ЮАР</x:v>
       </x:c>
       <x:c r="F28" s="77" t="str"/>
       <x:c r="G28" s="78" t="str"/>
       <x:c r="H28" s="79" t="str">
-        <x:v>Spain - Saudi Arabia
-Группа H · #37</x:v>
+        <x:v>Испания - Саудовская Аравия</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="43.5" customHeight="1">
@@ -1398,14 +1369,12 @@
       <x:c r="B29" s="77" t="str"/>
       <x:c r="C29" s="77" t="str"/>
       <x:c r="D29" s="79" t="str">
-        <x:v>Portugal - DR Congo
-Группа K · #21</x:v>
+        <x:v>Португалия - ДР Конго</x:v>
       </x:c>
       <x:c r="E29" s="77" t="str"/>
       <x:c r="F29" s="77" t="str"/>
       <x:c r="G29" s="79" t="str">
-        <x:v>Netherlands - Sweden
-Группа F · #33</x:v>
+        <x:v>Нидерланды - Швеция</x:v>
       </x:c>
       <x:c r="H29" s="78" t="str"/>
     </x:row>
@@ -1414,26 +1383,21 @@
         <x:v>22:00</x:v>
       </x:c>
       <x:c r="B30" s="79" t="str">
-        <x:v>Belgium - Egypt
-Группа G · #14</x:v>
+        <x:v>Бельгия - Египет</x:v>
       </x:c>
       <x:c r="C30" s="79" t="str">
-        <x:v>France - Senegal
-Группа I · #17</x:v>
+        <x:v>Франция - Сенегал</x:v>
       </x:c>
       <x:c r="D30" s="77" t="str"/>
       <x:c r="E30" s="79" t="str">
-        <x:v>Switzerland - Bosnia &amp; Herzegovina
-Группа B · #26</x:v>
+        <x:v>Швейцария - Босния и Герцеговина</x:v>
       </x:c>
       <x:c r="F30" s="79" t="str">
-        <x:v>USA - Australia
-Группа D · #29</x:v>
+        <x:v>США - Австралия</x:v>
       </x:c>
       <x:c r="G30" s="78" t="str"/>
       <x:c r="H30" s="79" t="str">
-        <x:v>Belgium - Iran
-Группа G · #38</x:v>
+        <x:v>Бельгия - Иран</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="43.5" customHeight="1">
@@ -1443,14 +1407,12 @@
       <x:c r="B31" s="77" t="str"/>
       <x:c r="C31" s="77" t="str"/>
       <x:c r="D31" s="79" t="str">
-        <x:v>England - Croatia
-Группа L · #22</x:v>
+        <x:v>Англия - Хорватия</x:v>
       </x:c>
       <x:c r="E31" s="77" t="str"/>
       <x:c r="F31" s="77" t="str"/>
       <x:c r="G31" s="79" t="str">
-        <x:v>Germany - Ivory Coast
-Группа E · #34</x:v>
+        <x:v>Германия - Кот-д’Ивуар</x:v>
       </x:c>
       <x:c r="H31" s="78" t="str"/>
     </x:row>
@@ -1556,18 +1518,15 @@
       </x:c>
       <x:c r="B37" s="77" t="str"/>
       <x:c r="C37" s="79" t="str">
-        <x:v>France - Iraq
-Группа I · #42</x:v>
+        <x:v>Франция - Ирак</x:v>
       </x:c>
       <x:c r="D37" s="77" t="str"/>
       <x:c r="E37" s="77" t="str"/>
       <x:c r="F37" s="77" t="str"/>
       <x:c r="G37" s="78" t="str"/>
       <x:c r="H37" s="80" t="str">
-        <x:v>Panama - England
-Группа L · #67
-Croatia - Ghana
-Группа L · #68</x:v>
+        <x:v>Панама - Англия
+Хорватия - Гана</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="69" customHeight="1">
@@ -1575,16 +1534,13 @@
         <x:v>01:00</x:v>
       </x:c>
       <x:c r="B38" s="79" t="str">
-        <x:v>Uruguay - Cape Verde
-Группа H · #39</x:v>
+        <x:v>Уругвай - Кабо-Верде</x:v>
       </x:c>
       <x:c r="C38" s="77" t="str"/>
       <x:c r="D38" s="77" t="str"/>
       <x:c r="E38" s="80" t="str">
-        <x:v>Scotland - Brazil
-Группа C · #51
-Morocco - Haiti
-Группа C · #52</x:v>
+        <x:v>Шотландия - Бразилия
+Марокко - Гаити</x:v>
       </x:c>
       <x:c r="F38" s="77" t="str"/>
       <x:c r="G38" s="78" t="str"/>
@@ -1597,15 +1553,12 @@
       <x:c r="B39" s="77" t="str"/>
       <x:c r="C39" s="77" t="str"/>
       <x:c r="D39" s="79" t="str">
-        <x:v>Panama - Croatia
-Группа L · #47</x:v>
+        <x:v>Панама - Хорватия</x:v>
       </x:c>
       <x:c r="E39" s="77" t="str"/>
       <x:c r="F39" s="80" t="str">
-        <x:v>Japan - Sweden
-Группа F · #57
-Tunisia - Netherlands
-Группа F · #58</x:v>
+        <x:v>Япония - Швеция
+Тунис - Нидерланды</x:v>
       </x:c>
       <x:c r="G39" s="78" t="str"/>
       <x:c r="H39" s="78" t="str"/>
@@ -1621,10 +1574,8 @@
       <x:c r="F40" s="77" t="str"/>
       <x:c r="G40" s="78" t="str"/>
       <x:c r="H40" s="80" t="str">
-        <x:v>Colombia - Portugal
-Группа K · #69
-DR Congo - Uzbekistan
-Группа K · #70</x:v>
+        <x:v>Колумбия - Португалия
+ДР Конго - Узбекистан</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="69" customHeight="1">
@@ -1633,17 +1584,14 @@
       </x:c>
       <x:c r="B41" s="77" t="str"/>
       <x:c r="C41" s="79" t="str">
-        <x:v>Norway - Senegal
-Группа I · #43</x:v>
+        <x:v>Норвегия - Сенегал</x:v>
       </x:c>
       <x:c r="D41" s="77" t="str"/>
       <x:c r="E41" s="77" t="str"/>
       <x:c r="F41" s="77" t="str"/>
       <x:c r="G41" s="80" t="str">
-        <x:v>Cape Verde - Saudi Arabia
-Группа H · #63
-Uruguay - Spain
-Группа H · #64</x:v>
+        <x:v>Кабо-Верде - Саудовская Аравия
+Уругвай - Испания</x:v>
       </x:c>
       <x:c r="H41" s="78" t="str"/>
     </x:row>
@@ -1652,16 +1600,13 @@
         <x:v>04:00</x:v>
       </x:c>
       <x:c r="B42" s="79" t="str">
-        <x:v>New Zealand - Egypt
-Группа G · #40</x:v>
+        <x:v>Новая Зеландия - Египет</x:v>
       </x:c>
       <x:c r="C42" s="77" t="str"/>
       <x:c r="D42" s="77" t="str"/>
       <x:c r="E42" s="80" t="str">
-        <x:v>Czechia - Mexico
-Группа A · #53
-South Africa - South Korea
-Группа A · #54</x:v>
+        <x:v>Чехия - Мексика
+ЮАР - Южная Корея</x:v>
       </x:c>
       <x:c r="F42" s="77" t="str"/>
       <x:c r="G42" s="78" t="str"/>
@@ -1674,22 +1619,17 @@
       <x:c r="B43" s="77" t="str"/>
       <x:c r="C43" s="77" t="str"/>
       <x:c r="D43" s="79" t="str">
-        <x:v>Colombia - DR Congo
-Группа K · #48</x:v>
+        <x:v>Колумбия - ДР Конго</x:v>
       </x:c>
       <x:c r="E43" s="77" t="str"/>
       <x:c r="F43" s="80" t="str">
-        <x:v>Türkiye - USA
-Группа D · #59
-Paraguay - Australia
-Группа D · #60</x:v>
+        <x:v>Турция - США
+Парагвай - Австралия</x:v>
       </x:c>
       <x:c r="G43" s="78" t="str"/>
       <x:c r="H43" s="80" t="str">
-        <x:v>Algeria - Austria
-Группа J · #71
-Jordan - Argentina
-Группа J · #72</x:v>
+        <x:v>Алжир - Австрия
+Иордания - Аргентина</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="69" customHeight="1">
@@ -1698,17 +1638,14 @@
       </x:c>
       <x:c r="B44" s="77" t="str"/>
       <x:c r="C44" s="79" t="str">
-        <x:v>Jordan - Algeria
-Группа J · #44</x:v>
+        <x:v>Иордания - Алжир</x:v>
       </x:c>
       <x:c r="D44" s="77" t="str"/>
       <x:c r="E44" s="77" t="str"/>
       <x:c r="F44" s="77" t="str"/>
       <x:c r="G44" s="80" t="str">
-        <x:v>Egypt - Iran
-Группа G · #65
-New Zealand - Belgium
-Группа G · #66</x:v>
+        <x:v>Египет - Иран
+Новая Зеландия - Бельгия</x:v>
       </x:c>
       <x:c r="H44" s="78" t="str"/>
     </x:row>
@@ -1717,12 +1654,10 @@
         <x:v>20:00</x:v>
       </x:c>
       <x:c r="B45" s="79" t="str">
-        <x:v>Argentina - Austria
-Группа J · #41</x:v>
+        <x:v>Аргентина - Австрия</x:v>
       </x:c>
       <x:c r="C45" s="79" t="str">
-        <x:v>Portugal - Uzbekistan
-Группа K · #45</x:v>
+        <x:v>Португалия - Узбекистан</x:v>
       </x:c>
       <x:c r="D45" s="77" t="str"/>
       <x:c r="E45" s="77" t="str"/>
@@ -1737,22 +1672,17 @@
       <x:c r="B46" s="77" t="str"/>
       <x:c r="C46" s="77" t="str"/>
       <x:c r="D46" s="80" t="str">
-        <x:v>Switzerland - Canada
-Группа B · #49
-Bosnia &amp; Herzegovina - Qatar
-Группа B · #50</x:v>
+        <x:v>Швейцария - Канада
+Босния и Герцеговина - Катар</x:v>
       </x:c>
       <x:c r="E46" s="77" t="str"/>
       <x:c r="F46" s="80" t="str">
-        <x:v>Norway - France
-Группа I · #61
-Senegal - Iraq
-Группа I · #62</x:v>
+        <x:v>Норвегия - Франция
+Сенегал - Ирак</x:v>
       </x:c>
       <x:c r="G46" s="78" t="str"/>
       <x:c r="H46" s="81" t="str">
-        <x:v>Runner-up A - Runner-up B
-1/16 финала · #73</x:v>
+        <x:v>2-е место группы A - 2-е место группы B</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="69" customHeight="1">
@@ -1761,15 +1691,12 @@
       </x:c>
       <x:c r="B47" s="77" t="str"/>
       <x:c r="C47" s="79" t="str">
-        <x:v>England - Ghana
-Группа L · #46</x:v>
+        <x:v>Англия - Гана</x:v>
       </x:c>
       <x:c r="D47" s="77" t="str"/>
       <x:c r="E47" s="80" t="str">
-        <x:v>Curaçao - Ivory Coast
-Группа E · #55
-Ecuador - Germany
-Группа E · #56</x:v>
+        <x:v>Кюрасао - Кот-д’Ивуар
+Эквадор - Германия</x:v>
       </x:c>
       <x:c r="F47" s="77" t="str"/>
       <x:c r="G47" s="78" t="str"/>
@@ -1878,15 +1805,13 @@
       <x:c r="B53" s="77" t="str"/>
       <x:c r="C53" s="77" t="str"/>
       <x:c r="D53" s="81" t="str">
-        <x:v>Winner I - Best 3rd (C/D/F/G/H)
-1/16 финала · #78</x:v>
+        <x:v>Победитель группы I - Лучшая 3-я команда (C/D/F/G/H)</x:v>
       </x:c>
       <x:c r="E53" s="77" t="str"/>
       <x:c r="F53" s="77" t="str"/>
       <x:c r="G53" s="78" t="str"/>
       <x:c r="H53" s="81" t="str">
-        <x:v>W74 - W77
-1/8 финала · #89</x:v>
+        <x:v>Победитель матча 74 - Победитель матча 77</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="43.5" customHeight="1">
@@ -1899,8 +1824,7 @@
       <x:c r="E54" s="77" t="str"/>
       <x:c r="F54" s="77" t="str"/>
       <x:c r="G54" s="81" t="str">
-        <x:v>Winner J - Runner-up H
-1/16 финала · #87</x:v>
+        <x:v>Победитель группы J - 2-е место группы H</x:v>
       </x:c>
       <x:c r="H54" s="78" t="str"/>
     </x:row>
@@ -1913,8 +1837,7 @@
       <x:c r="D55" s="77" t="str"/>
       <x:c r="E55" s="77" t="str"/>
       <x:c r="F55" s="81" t="str">
-        <x:v>Runner-up K - Runner-up L
-1/16 финала · #84</x:v>
+        <x:v>2-е место группы K - 2-е место группы L</x:v>
       </x:c>
       <x:c r="G55" s="78" t="str"/>
       <x:c r="H55" s="78" t="str"/>
@@ -1927,8 +1850,7 @@
       <x:c r="C56" s="77" t="str"/>
       <x:c r="D56" s="77" t="str"/>
       <x:c r="E56" s="81" t="str">
-        <x:v>Winner D - Best 3rd (B/E/F/I/J)
-1/16 финала · #82</x:v>
+        <x:v>Победитель группы D - Лучшая 3-я команда (B/E/F/I/J)</x:v>
       </x:c>
       <x:c r="F56" s="77" t="str"/>
       <x:c r="G56" s="78" t="str"/>
@@ -1940,12 +1862,10 @@
       </x:c>
       <x:c r="B57" s="77" t="str"/>
       <x:c r="C57" s="81" t="str">
-        <x:v>Winner F - Runner-up C
-1/16 финала · #76</x:v>
+        <x:v>Победитель группы F - 2-е место группы C</x:v>
       </x:c>
       <x:c r="D57" s="81" t="str">
-        <x:v>Winner A - Best 3rd (C/E/F/H/I)
-1/16 финала · #79</x:v>
+        <x:v>Победитель группы A - Лучшая 3-я команда (C/E/F/H/I)</x:v>
       </x:c>
       <x:c r="E57" s="77" t="str"/>
       <x:c r="F57" s="77" t="str"/>
@@ -1962,8 +1882,7 @@
       <x:c r="E58" s="77" t="str"/>
       <x:c r="F58" s="77" t="str"/>
       <x:c r="G58" s="81" t="str">
-        <x:v>Winner K - Best 3rd (D/E/I/J/L)
-1/16 финала · #88</x:v>
+        <x:v>Победитель группы K - Лучшая 3-я команда (D/E/I/J/L)</x:v>
       </x:c>
       <x:c r="H58" s="78" t="str"/>
     </x:row>
@@ -1976,8 +1895,7 @@
       <x:c r="D59" s="77" t="str"/>
       <x:c r="E59" s="77" t="str"/>
       <x:c r="F59" s="81" t="str">
-        <x:v>Winner B - Best 3rd (E/F/G/I/J)
-1/16 финала · #85</x:v>
+        <x:v>Победитель группы B - Лучшая 3-я команда (E/F/G/I/J)</x:v>
       </x:c>
       <x:c r="G59" s="78" t="str"/>
       <x:c r="H59" s="78" t="str"/>
@@ -1989,8 +1907,7 @@
       <x:c r="B60" s="77" t="str"/>
       <x:c r="C60" s="77" t="str"/>
       <x:c r="D60" s="81" t="str">
-        <x:v>Winner L - Best 3rd (E/H/I/J/K)
-1/16 финала · #80</x:v>
+        <x:v>Победитель группы L - Лучшая 3-я команда (E/H/I/J/K)</x:v>
       </x:c>
       <x:c r="E60" s="77" t="str"/>
       <x:c r="F60" s="77" t="str"/>
@@ -2002,19 +1919,16 @@
         <x:v>20:00</x:v>
       </x:c>
       <x:c r="B61" s="81" t="str">
-        <x:v>Winner C - Runner-up F
-1/16 финала · #74</x:v>
+        <x:v>Победитель группы C - 2-е место группы F</x:v>
       </x:c>
       <x:c r="C61" s="81" t="str">
-        <x:v>Runner-up E - Runner-up I
-1/16 финала · #77</x:v>
+        <x:v>2-е место группы E - 2-е место группы I</x:v>
       </x:c>
       <x:c r="D61" s="77" t="str"/>
       <x:c r="E61" s="77" t="str"/>
       <x:c r="F61" s="77" t="str"/>
       <x:c r="G61" s="81" t="str">
-        <x:v>W73 - W75
-1/8 финала · #90</x:v>
+        <x:v>Победитель матча 73 - Победитель матча 75</x:v>
       </x:c>
       <x:c r="H61" s="78" t="str"/>
     </x:row>
@@ -2027,8 +1941,7 @@
       <x:c r="D62" s="77" t="str"/>
       <x:c r="E62" s="77" t="str"/>
       <x:c r="F62" s="81" t="str">
-        <x:v>Runner-up D - Runner-up G
-1/16 финала · #86</x:v>
+        <x:v>2-е место группы D - 2-е место группы G</x:v>
       </x:c>
       <x:c r="G62" s="78" t="str"/>
       <x:c r="H62" s="78" t="str"/>
@@ -2041,8 +1954,7 @@
       <x:c r="C63" s="77" t="str"/>
       <x:c r="D63" s="77" t="str"/>
       <x:c r="E63" s="81" t="str">
-        <x:v>Winner H - Runner-up J
-1/16 финала · #83</x:v>
+        <x:v>Победитель группы H - 2-е место группы J</x:v>
       </x:c>
       <x:c r="F63" s="77" t="str"/>
       <x:c r="G63" s="78" t="str"/>
@@ -2055,15 +1967,13 @@
       <x:c r="B64" s="77" t="str"/>
       <x:c r="C64" s="77" t="str"/>
       <x:c r="D64" s="81" t="str">
-        <x:v>Winner G - Best 3rd (A/E/H/I/J)
-1/16 финала · #81</x:v>
+        <x:v>Победитель группы G - Лучшая 3-я команда (A/E/H/I/J)</x:v>
       </x:c>
       <x:c r="E64" s="77" t="str"/>
       <x:c r="F64" s="77" t="str"/>
       <x:c r="G64" s="78" t="str"/>
       <x:c r="H64" s="81" t="str">
-        <x:v>W76 - W78
-1/8 финала · #91</x:v>
+        <x:v>Победитель матча 76 - Победитель матча 78</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="43.5" customHeight="1">
@@ -2071,8 +1981,7 @@
         <x:v>23:30</x:v>
       </x:c>
       <x:c r="B65" s="81" t="str">
-        <x:v>Winner E - Best 3rd (A/B/C/D/F)
-1/16 финала · #75</x:v>
+        <x:v>Победитель группы E - Лучшая 3-я команда (A/B/C/D/F)</x:v>
       </x:c>
       <x:c r="C65" s="77" t="str"/>
       <x:c r="D65" s="77" t="str"/>
@@ -2188,8 +2097,7 @@
       <x:c r="F71" s="77" t="str"/>
       <x:c r="G71" s="78" t="str"/>
       <x:c r="H71" s="81" t="str">
-        <x:v>W91 - W92
-Четвертьфинал · #99</x:v>
+        <x:v>Победитель матча 91 - Победитель матча 92</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="43.5" customHeight="1">
@@ -2197,12 +2105,10 @@
         <x:v>03:00</x:v>
       </x:c>
       <x:c r="B72" s="81" t="str">
-        <x:v>W79 - W80
-1/8 финала · #92</x:v>
+        <x:v>Победитель матча 79 - Победитель матча 80</x:v>
       </x:c>
       <x:c r="C72" s="81" t="str">
-        <x:v>W81 - W82
-1/8 финала · #94</x:v>
+        <x:v>Победитель матча 81 - Победитель матча 82</x:v>
       </x:c>
       <x:c r="D72" s="77" t="str"/>
       <x:c r="E72" s="77" t="str"/>
@@ -2221,8 +2127,7 @@
       <x:c r="F73" s="77" t="str"/>
       <x:c r="G73" s="78" t="str"/>
       <x:c r="H73" s="81" t="str">
-        <x:v>W95 - W96
-Четвертьфинал · #100</x:v>
+        <x:v>Победитель матча 95 - Победитель матча 96</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="43.5" customHeight="1">
@@ -2231,8 +2136,7 @@
       </x:c>
       <x:c r="B74" s="77" t="str"/>
       <x:c r="C74" s="81" t="str">
-        <x:v>W86 - W88
-1/8 финала · #95</x:v>
+        <x:v>Победитель матча 86 - Победитель матча 88</x:v>
       </x:c>
       <x:c r="D74" s="77" t="str"/>
       <x:c r="E74" s="77" t="str"/>
@@ -2245,15 +2149,13 @@
         <x:v>22:00</x:v>
       </x:c>
       <x:c r="B75" s="81" t="str">
-        <x:v>W83 - W84
-1/8 финала · #93</x:v>
+        <x:v>Победитель матча 83 - Победитель матча 84</x:v>
       </x:c>
       <x:c r="C75" s="77" t="str"/>
       <x:c r="D75" s="77" t="str"/>
       <x:c r="E75" s="77" t="str"/>
       <x:c r="F75" s="81" t="str">
-        <x:v>W93 - W94
-Четвертьфинал · #98</x:v>
+        <x:v>Победитель матча 93 - Победитель матча 94</x:v>
       </x:c>
       <x:c r="G75" s="78" t="str"/>
       <x:c r="H75" s="78" t="str"/>
@@ -2264,13 +2166,11 @@
       </x:c>
       <x:c r="B76" s="77" t="str"/>
       <x:c r="C76" s="81" t="str">
-        <x:v>W85 - W87
-1/8 финала · #96</x:v>
+        <x:v>Победитель матча 85 - Победитель матча 87</x:v>
       </x:c>
       <x:c r="D76" s="77" t="str"/>
       <x:c r="E76" s="81" t="str">
-        <x:v>W89 - W90
-Четвертьфинал · #97</x:v>
+        <x:v>Победитель матча 89 - Победитель матча 90</x:v>
       </x:c>
       <x:c r="F76" s="77" t="str"/>
       <x:c r="G76" s="78" t="str"/>
@@ -2383,8 +2283,7 @@
       <x:c r="F82" s="77" t="str"/>
       <x:c r="G82" s="78" t="str"/>
       <x:c r="H82" s="81" t="str">
-        <x:v>L101 - L102
-Матч за 3 место · #103</x:v>
+        <x:v>Проигравший матча 101 - Проигравший матча 102</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="43.5" customHeight="1">
@@ -2393,19 +2292,16 @@
       </x:c>
       <x:c r="B83" s="77" t="str"/>
       <x:c r="C83" s="81" t="str">
-        <x:v>W97 - W98
-Полуфинал · #101</x:v>
+        <x:v>Победитель матча 97 - Победитель матча 98</x:v>
       </x:c>
       <x:c r="D83" s="81" t="str">
-        <x:v>W99 - W100
-Полуфинал · #102</x:v>
+        <x:v>Победитель матча 99 - Победитель матча 100</x:v>
       </x:c>
       <x:c r="E83" s="77" t="str"/>
       <x:c r="F83" s="77" t="str"/>
       <x:c r="G83" s="78" t="str"/>
       <x:c r="H83" s="81" t="str">
-        <x:v>W101 - W102
-Финал · #104</x:v>
+        <x:v>Победитель матча 101 - Победитель матча 102</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5611,7 +5507,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red69baed2048476b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46294929077a4c0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9837,7 +9733,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra41cb5047b0f4070"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf4c85171f9640bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10277,9 +10173,9 @@
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b753777fdf142d9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06fbd27b1f1041e8"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b7df382d7504179"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf68269ab88a6472c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10623,7 +10519,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R749e3201b2bf44bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad49b114c312425c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>